<commit_message>
fix(eckr): UK-only rebuild - all 36 competitors verified UK-located
Re-scraped all 9 categories with a UK-location filter (search-card 'from
<country>' + per-listing 'Located in'); removed US/China listings that slipped
past eBay's LH_PrefLoc filter (entire Pipe/Spider categories were foreign).
36 UK-verified rows (Pipe/Spider collapse to 1 each - almost no UK competition).
Rebuilt dashboard/static/xlsx; re-published to ph_task 496-499 (read-back 58114).
Shipping left as-is per Abiraj (UK shipping not reliably readable from LK IP).
</commit_message>
<xml_diff>
--- a/development/abiraj_mini_aios_workbench/projects/PRJ-2026-017_ebay-competitor-keyword-research/evidence/final_outputs/REQ-20_ebay-competitor-keyword-research/REQ-20-D01_ebay_competitor_keyword_FINAL.xlsx
+++ b/development/abiraj_mini_aios_workbench/projects/PRJ-2026-017_ebay-competitor-keyword-research/evidence/final_outputs/REQ-20_ebay-competitor-keyword-research/REQ-20-D01_ebay_competitor_keyword_FINAL.xlsx
@@ -1031,156 +1031,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId36"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>37</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="37" name="Image 37" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId37"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>38</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="38" name="Image 38" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId38"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>39</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="39" name="Image 39" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId39"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>40</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="40" name="Image 40" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>41</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="41" name="Image 41" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId41"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>42</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="609600" cy="609600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="42" name="Image 42" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId42"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1483,7 +1333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:N37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1647,32 +1497,32 @@
       <c r="B3" s="2" t="inlineStr"/>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>333667118358</t>
+          <t>113986270784</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>firstchoicelighting</t>
+          <t>Country Club</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Set of 2 Modern Black Metal Swirl Easy Fit Ceiling Light Shade</t>
+          <t>Gem Wrap Twist Design Glamour Silver Metal Lamp Shade Easy Fit</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>268</t>
+          <t>317</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>GBP  23.45</t>
+          <t>GBP  118.95</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>99.7% (89.9K)</t>
+          <t>99.5% (136.8K)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -1686,7 +1536,7 @@
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: firstchoicelightingoutlet</t>
+          <t>Competitor seller: eshhopinguk</t>
         </is>
       </c>
     </row>
@@ -1695,32 +1545,32 @@
       <c r="B4" s="2" t="inlineStr"/>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>285423964421</t>
+          <t>333667118358</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Giggi</t>
+          <t>firstchoicelighting</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Metal &amp; Rope Lamp Shades Ceiling Pendant Light Shade</t>
+          <t>Set of 2 Modern Black Metal Swirl Easy Fit Ceiling Light Shade</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>268</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>GBP  18.99</t>
+          <t>GBP  23.45</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>99.6% (21.9K)</t>
+          <t>99.7% (89.9K)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -1728,17 +1578,13 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Save up to 15% Multi-buy</t>
-        </is>
-      </c>
+      <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: picknmix.online</t>
+          <t>Competitor seller: firstchoicelightingoutlet</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1618,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>99.8% (26.7K)</t>
+          <t>99.8% (26.8K)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -1799,32 +1645,32 @@
       <c r="B6" s="2" t="inlineStr"/>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>163799621837</t>
+          <t>202880784935</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>Optimal Products</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Lampshade Industrial Pendant Ceiling Light Silver Metal Retro Nordic</t>
+          <t>Silver Gem Wrap Twist Design Pendant Glamour Metal Lamp Shade</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>19+</t>
+          <t>38</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>GBP  14.00 to 29.00</t>
+          <t>GBP  118.95</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>100% (3.1K)</t>
+          <t>99.7% (220.4K)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -1838,7 +1684,7 @@
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: goodwood-originals123</t>
+          <t>Competitor seller: buybox786</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1707,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Vintage Industrial Wall Light Antique Retro Cage Bulkhead Gold Brass Ship Lamp</t>
+          <t>Vintage Industrial Wall Light Antique Retro Cage Bulkhead Gold Brass</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1911,32 +1757,32 @@
       <c r="B8" s="2" t="inlineStr"/>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>234566652967</t>
+          <t>353351065595</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>(not listed)</t>
+          <t>ValueLights</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Vintage Industrial Wall Light Antique Retro Style Lamp Sconce Fixture Rustic</t>
+          <t>Industrial Style Wall Light Polished Chrome with Glass Shades</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>180+</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>GBP  31.99</t>
+          <t>GBP  26.99 to 29.99</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>99.7% (9.8K)</t>
+          <t>99.8% (685K)</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -1944,13 +1790,17 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>From GBP 18.89 with coupon</t>
+        </is>
+      </c>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: burgesshandg</t>
+          <t>Competitor seller: value-lights</t>
         </is>
       </c>
     </row>
@@ -1959,32 +1809,32 @@
       <c r="B9" s="2" t="inlineStr"/>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>155030374927</t>
+          <t>234566652967</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>(not listed)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Modern Vintage Retro Industrial Rustic Sconce Wall Light</t>
+          <t>Vintage Industrial Wall Light Antique Retro Style Lamp Sconce</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>71</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>GBP  7.99</t>
+          <t>GBP  31.99</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>99.7% (5.5K)</t>
+          <t>99.7% (9.8K)</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1992,17 +1842,13 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>Save up to 6% Multi-buy</t>
-        </is>
-      </c>
+      <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: theyinltd</t>
+          <t>Competitor seller: burgesshandg</t>
         </is>
       </c>
     </row>
@@ -2011,32 +1857,32 @@
       <c r="B10" s="2" t="inlineStr"/>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>116478119802</t>
+          <t>256403363785</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>(not listed)</t>
+          <t>Davey &amp; Co</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Industrial Bulkhead Light Wall Ceiling Retro Old Marine Brass Gold</t>
+          <t>Davey &amp; Co Style Industrial Bulkhead Wall Light Vintage Antique</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>57</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>GBP  69.99</t>
+          <t>GBP  57.99</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>100% (1.4K)</t>
+          <t>98.5% (15.2K)</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -2050,7 +1896,7 @@
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: eat_sleep_buy_repeat</t>
+          <t>Competitor seller: sj_modern_antiques</t>
         </is>
       </c>
     </row>
@@ -2059,32 +1905,32 @@
       <c r="B11" s="2" t="inlineStr"/>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>137354830445</t>
+          <t>364433876601</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Does not apply</t>
+          <t>(not listed)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Vintage Brass Boho Wall Sconces with Tulip Glass Shade for Modern Spaces</t>
+          <t>Outdoor Vintage Replica Industrial Round Caged IP44 Bulkhead Wall Light</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>56</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>GBP  81.26</t>
+          <t>GBP  12.99</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>99.8% (28.1K)</t>
+          <t>99.6% (410.1K)</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -2098,7 +1944,7 @@
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: weshipnow</t>
+          <t>Competitor seller: discountcdrom</t>
         </is>
       </c>
     </row>
@@ -2121,7 +1967,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Ceiling Light Fitting 3 Way Chrome Spotlight Swirl Glass</t>
+          <t>Ceiling Light Fitting 3 Way Chrome Spotlight Swirl</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -2171,32 +2017,32 @@
       <c r="B13" s="2" t="inlineStr"/>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>372336415252</t>
+          <t>333667118358</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>ValueLights</t>
+          <t>firstchoicelighting</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Lampshade Ceiling Pendant Light Shade Easy Fit Chandelier</t>
+          <t>Set of 2 Modern Black Metal Swirl Easy Fit Ceiling Light Shade</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>6,442+</t>
+          <t>268</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>GBP  17.99</t>
+          <t>GBP  23.45</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>99.8% (685K)</t>
+          <t>99.7% (89.9K)</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -2204,17 +2050,13 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>Save up to 10% Multi-buy</t>
-        </is>
-      </c>
+      <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: value-lights</t>
+          <t>Competitor seller: firstchoicelightingoutlet</t>
         </is>
       </c>
     </row>
@@ -2223,32 +2065,32 @@
       <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>333667118358</t>
+          <t>405002496188</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>firstchoicelighting</t>
+          <t>Homion</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Set of 2 Modern Black Metal Swirl Easy Fit Ceiling Light Shade</t>
+          <t>Ancient Moroccan Style Metal Ceiling Light Shade Easy Fit Pendant</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>268</t>
+          <t>61+</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>GBP  23.45</t>
+          <t>GBP  99.99</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>99.7% (89.9K)</t>
+          <t>99.8% (26.8K)</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -2256,13 +2098,17 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Save up to 6% Multi-buy</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: firstchoicelightingoutlet</t>
+          <t>Competitor seller: online336</t>
         </is>
       </c>
     </row>
@@ -2271,32 +2117,32 @@
       <c r="B15" s="2" t="inlineStr"/>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>285423964421</t>
+          <t>154043319055</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Giggi</t>
+          <t>Innoteck</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Metal &amp; Rope Lamp Shades Ceiling Pendant Light Shade</t>
+          <t>Metal Drum Vintage Light Shade Modern Decorative Ceiling Pendant</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>58+</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>GBP  18.99</t>
+          <t>GBP  14.99</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>99.6% (21.9K)</t>
+          <t>99.9% (60.1K)</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -2304,17 +2150,13 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>Save up to 15% Multi-buy</t>
-        </is>
-      </c>
+      <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: picknmix.online</t>
+          <t>Competitor seller: homeessenceltd</t>
         </is>
       </c>
     </row>
@@ -2323,32 +2165,32 @@
       <c r="B16" s="2" t="inlineStr"/>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>393696656791</t>
+          <t>163799621837</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Innoteck</t>
+          <t>Unbranded</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Innoteck Ceiling Light Shade - Modern Chandelier Pendant</t>
+          <t>Lampshade Industrial Pendant Ceiling Light Silver Metal Retro Nordic</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>92+</t>
+          <t>19+</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>GBP  10.49</t>
+          <t>GBP  14.00 to 29.00</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>99.8% (10.2K)</t>
+          <t>100% (3.1K)</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -2356,17 +2198,13 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Save up to 20% Multi-buy</t>
-        </is>
-      </c>
+      <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: innoteck_uk</t>
+          <t>Competitor seller: goodwood-originals123</t>
         </is>
       </c>
     </row>
@@ -2379,32 +2217,32 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>333675680799</t>
+          <t>372257187156</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>firstchoicelighting</t>
+          <t>ValueLights</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Set of 2 Modern Three Tier Easy Fit Jewelled Ceiling Light</t>
+          <t>Ceiling Light Fitting 3 Way Chrome Spotlight Swirl Glass</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>751</t>
+          <t>8,367</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>GBP  20.39</t>
+          <t>GBP  19.99</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>99.7% (89.9K)</t>
+          <t>99.8% (685K)</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -2430,7 +2268,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: firstchoicelightingoutlet</t>
+          <t>Competitor seller: value-lights</t>
         </is>
       </c>
     </row>
@@ -2487,32 +2325,32 @@
       <c r="B19" s="2" t="inlineStr"/>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>272110237788</t>
+          <t>141200077246</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>MoonLight Retail</t>
+          <t>ElekTek</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>New Modern Vintage Industrial Retro Loft Glass Ceiling Lamp Shade</t>
+          <t>ElekTek 3-Hook Ceiling Rose Pendant Plate Suspended Glass</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>269+</t>
+          <t>516+</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>GBP  32.47 to 35.83</t>
+          <t>GBP  17.25 to 19.99</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>100% (3.9K)</t>
+          <t>99.9% (55.5K)</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -2522,7 +2360,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Save up to 5% Multi-buy</t>
+          <t>Save up to 7% Multi-buy</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr"/>
@@ -2530,7 +2368,7 @@
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: moonlight_retail_15</t>
+          <t>Competitor seller: buyitbetter_uk</t>
         </is>
       </c>
     </row>
@@ -2539,32 +2377,32 @@
       <c r="B20" s="2" t="inlineStr"/>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>141200077246</t>
+          <t>272110237788</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>ElekTek</t>
+          <t>MoonLight Retail</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>ElekTek 3-Hook Ceiling Rose Pendant Plate Suspended Glass</t>
+          <t>New Modern Vintage Industrial Retro Loft Glass Ceiling Lamp Shade</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>59+</t>
+          <t>269+</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>GBP  17.25 to 19.99</t>
+          <t>GBP  32.47 to 35.83</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>99.9% (55.5K)</t>
+          <t>100% (3.9K)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -2574,7 +2412,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Save up to 7% Multi-buy</t>
+          <t>Save up to 5% Multi-buy</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
@@ -2582,7 +2420,7 @@
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: buyitbetter_uk</t>
+          <t>Competitor seller: moonlight_retail_15</t>
         </is>
       </c>
     </row>
@@ -2591,32 +2429,32 @@
       <c r="B21" s="2" t="inlineStr"/>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>356659461782</t>
+          <t>333667118358</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>ValueLights</t>
+          <t>firstchoicelighting</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Corinne Spiral Twill Glass Easy Fit Ceiling Pendant Light Shade</t>
+          <t>Set of 2 Modern Black Metal Swirl Easy Fit Ceiling Light Shade</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>268</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>GBP  34.99 to 37.99</t>
+          <t>GBP  23.45</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>99.8% (685K)</t>
+          <t>99.7% (89.9K)</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -2624,17 +2462,13 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>From GBP 31.49 with coupon</t>
-        </is>
-      </c>
+      <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: value-lights</t>
+          <t>Competitor seller: firstchoicelightingoutlet</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2481,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>303682816669</t>
+          <t>406427712394</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -2657,22 +2491,22 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Retro 4/6/8/10/12 Heads Mix-color Chandelier Spider Pendant Ceiling Light</t>
+          <t>Duplex Spider Fitting for Pendant Lamp Shades BC B22 Bayonet Cap</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>28</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>GBP  22.99 to 49.99</t>
+          <t>GBP  7.85</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>96.4% (14.7K)</t>
+          <t>100% (1.6K)</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -2698,41 +2532,45 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: best-love2010</t>
+          <t>Competitor seller: ulsltd</t>
         </is>
       </c>
     </row>
     <row r="23" ht="52" customHeight="1">
       <c r="A23" s="2" t="inlineStr"/>
-      <c r="B23" s="2" t="inlineStr"/>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Cage pendant light</t>
+        </is>
+      </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>303227195662</t>
+          <t>372257190104</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>(not listed)</t>
+          <t>ValueLights</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Adjustable Pendant Light Fitting Ceiling Rose E27 Industrial Spider Hanging Lamp</t>
+          <t>Ceiling Light Shade Geometric Pendant Lampshade Industrial</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>429+</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>GBP  13.42 to 59.92</t>
+          <t>GBP  12.99 to 15.99</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>99.6% (18.4K)</t>
+          <t>99.8% (685K)</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -2740,13 +2578,29 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Save up to 10% Multi-buy</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Cage Pendant Light, Cage Light, Metal Cage Pendant</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Industrial Cage Light, Wire Cage Pendant, Vintage Cage Lamp, Cage Ceiling Light</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>Black Metal Cage Pendant Light for Kitchen, Industrial Wire Cage Hanging Lamp E27, Vintage Cage Ceiling Light Fitting</t>
+        </is>
+      </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: nationallighting</t>
+          <t>Competitor seller: value-lights</t>
         </is>
       </c>
     </row>
@@ -2755,32 +2609,32 @@
       <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>292861051418</t>
+          <t>232708905363</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>ValueLights</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Vintage Edison Multiple Adjustable DIY Ceiling Spider Light</t>
+          <t>Industrial Metal Ceiling Pendant Light Shade Easy Fit</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>34+</t>
+          <t>289+</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>GBP  11.99 to 21.99</t>
+          <t>GBP  22.99 to 25.99</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>96.4% (14.7K)</t>
+          <t>99.8% (685K)</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -2788,13 +2642,17 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>From GBP 20.69 with coupon</t>
+        </is>
+      </c>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: best-love2010</t>
+          <t>Competitor seller: value-lights</t>
         </is>
       </c>
     </row>
@@ -2803,32 +2661,32 @@
       <c r="B25" s="2" t="inlineStr"/>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>236823130326</t>
+          <t>131173303482</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>ANWIO</t>
+          <t>Unbranded</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>ANWIO 6 Heads Spider Light Chandelier Pendant DIY Spider Rope</t>
+          <t>Black Wire Cage Light Shade Steel E27 Industrial Pendant</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>252</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>GBP  29.99</t>
+          <t>GBP  13.00</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>99.8% (13.4K)</t>
+          <t>99.8% (22.6K)</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -2842,45 +2700,41 @@
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: wowzer-uk</t>
+          <t>Competitor seller: thelampfactoryuk</t>
         </is>
       </c>
     </row>
     <row r="26" ht="52" customHeight="1">
       <c r="A26" s="2" t="inlineStr"/>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Cage pendant light</t>
-        </is>
-      </c>
+      <c r="B26" s="2" t="inlineStr"/>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>372257190104</t>
+          <t>141264804458</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>ValueLights</t>
+          <t>Unbranded</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Ceiling Light Shade Geometric Pendant Lampshade Lamp Industrial</t>
+          <t>Bronze Wire Cage Light Shade Steel E27 Industrial Pendant</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>951+</t>
+          <t>157</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>GBP  12.99 to 15.99</t>
+          <t>GBP  13.00</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>99.8% (685K)</t>
+          <t>99.8% (22.6K)</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2888,63 +2742,51 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>Save up to 10% Multi-buy</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>Cage Pendant Light, Cage Light, Metal Cage Pendant</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>Industrial Cage Light, Wire Cage Pendant, Vintage Cage Lamp, Cage Ceiling Light</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="inlineStr">
-        <is>
-          <t>Black Metal Cage Pendant Light for Kitchen, Industrial Wire Cage Hanging Lamp E27, Vintage Cage Ceiling Light Fitting</t>
-        </is>
-      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: value-lights</t>
+          <t>Competitor seller: thelampfactoryuk</t>
         </is>
       </c>
     </row>
     <row r="27" ht="52" customHeight="1">
       <c r="A27" s="2" t="inlineStr"/>
-      <c r="B27" s="2" t="inlineStr"/>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Pipe Light</t>
+        </is>
+      </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>232708905363</t>
+          <t>262744851290</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>ValueLights</t>
+          <t>(not listed)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Industrial Metal Ceiling Pendant Light Shade Easy Fit</t>
+          <t>Silver Industrial Ceiling Light Vintage Antique Pendant Pipe Cage</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>289+</t>
+          <t>114</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>GBP  22.99 to 25.99</t>
+          <t>GBP  46.99</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>99.8% (685K)</t>
+          <t>98.5% (15.2K)</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -2952,51 +2794,63 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>From GBP 20.69 with coupon</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Pipe Light, Pipe Pendant Light, Steampunk Light</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Industrial Pipe Light, Steampunk Pendant, Pipe Wall Light, Water Pipe Lamp</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>Industrial Steampunk Pipe Pendant Light for Kitchen Island, Black Metal Pipe Ceiling Light E27, Vintage Water Pipe Wall Lamp</t>
+        </is>
+      </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: value-lights</t>
+          <t>Competitor seller: sj_modern_antiques</t>
         </is>
       </c>
     </row>
     <row r="28" ht="52" customHeight="1">
       <c r="A28" s="2" t="inlineStr"/>
-      <c r="B28" s="2" t="inlineStr"/>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Bulbs</t>
+        </is>
+      </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>131173303482</t>
+          <t>303695648760</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>Kanlux</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Black Wire Cage Light Shade Steel E27 Industrial Pendant</t>
+          <t>2x Vintage Filament LED Edison Screw Bulb E27 Decorative ST64</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>252</t>
+          <t>237</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>GBP  13.00</t>
+          <t>GBP  16.95</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>99.8% (22.6K)</t>
+          <t>99.7% (84.9K)</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -3004,13 +2858,29 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Save up to 20% Multi-buy</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>LED Bulb, Filament Bulb, Light Bulb</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Edison Bulb, Vintage LED Bulb, E27 Bulb, Dimmable LED Filament Bulb</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>E27 Vintage Edison LED Filament Bulb Warm White, Dimmable Squirrel Cage Light Bulb, ST64 Amber Decorative LED Bulb 4W</t>
+        </is>
+      </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: thelampfactoryuk</t>
+          <t>Competitor seller: auctionzltd</t>
         </is>
       </c>
     </row>
@@ -3019,32 +2889,32 @@
       <c r="B29" s="2" t="inlineStr"/>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>141264804458</t>
+          <t>223224109836</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>Auraglow</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Bronze Wire Cage Light Shade Steel E27 Industrial Pendant</t>
+          <t>Auraglow Mysa LED Light Bulb Vintage Retro Edison Style E27 T30</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>180</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>GBP  13.00</t>
+          <t>GBP  10.99</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>99.8% (22.6K)</t>
+          <t>99.8% (188.5K)</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -3058,7 +2928,7 @@
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: thelampfactoryuk</t>
+          <t>Competitor seller: safield-online</t>
         </is>
       </c>
     </row>
@@ -3067,32 +2937,32 @@
       <c r="B30" s="2" t="inlineStr"/>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>262744851290</t>
+          <t>142340181955</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>(not listed)</t>
+          <t>Unbranded</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Silver Industrial Ceiling Light Vintage Antique Pendant Cage</t>
+          <t>Vintage Edison Filament LED Bulb Teardrop E27 ES 4W Warm White</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>169</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>GBP  46.99</t>
+          <t>GBP  3.50</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>98.5% (15.2K)</t>
+          <t>99.8% (22.6K)</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -3106,45 +2976,41 @@
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: sj_modern_antiques</t>
+          <t>Competitor seller: thelampfactoryuk</t>
         </is>
       </c>
     </row>
     <row r="31" ht="52" customHeight="1">
       <c r="A31" s="2" t="inlineStr"/>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Pipe Light</t>
-        </is>
-      </c>
+      <c r="B31" s="2" t="inlineStr"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>174650219163</t>
+          <t>193185894331</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Stout &amp; Burg Designs</t>
+          <t>Auraglow</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Steampunk Industrial Iron Pipe Ceiling Light Pendant Kit</t>
+          <t>Auraglow Mysa LED Light Bulb Vintage Retro Edison Style G125 Globe</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>334+</t>
+          <t>156+</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>GBP  3.18 to 10.46</t>
+          <t>GBP  16.99</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>99% (4.4K)</t>
+          <t>99.8% (188.5K)</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -3153,24 +3019,12 @@
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>Pipe Light, Pipe Pendant Light, Steampunk Light</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>Industrial Pipe Light, Steampunk Pendant, Pipe Wall Light, Water Pipe Lamp</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="inlineStr">
-        <is>
-          <t>Industrial Steampunk Pipe Pendant Light for Kitchen Island, Black Metal Pipe Ceiling Light E27, Vintage Water Pipe Wall Lamp</t>
-        </is>
-      </c>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: nmstoute</t>
+          <t>Competitor seller: safield-online</t>
         </is>
       </c>
     </row>
@@ -3179,80 +3033,88 @@
       <c r="B32" s="2" t="inlineStr"/>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>353005301113</t>
+          <t>353206988280</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>Kanlux</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Iron Vintage Steampunk Industrial Pipe Ceiling Pendant Light</t>
+          <t>E27 LED Vintage Edison Spiral Filament Industrial Bulb Amber</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>128</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>GBP  16.22</t>
+          <t>GBP  7.95</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>99.4% (3K)</t>
+          <t>99.7% (84.9K)</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Free postage</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr"/>
+          <t>With postage</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Save up to 12% Multi-buy</t>
+        </is>
+      </c>
       <c r="K32" s="2" t="inlineStr"/>
       <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr"/>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: happy_home_2019</t>
+          <t>Competitor seller: auctionzltd</t>
         </is>
       </c>
     </row>
     <row r="33" ht="52" customHeight="1">
       <c r="A33" s="2" t="inlineStr"/>
-      <c r="B33" s="2" t="inlineStr"/>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Lamp Holder</t>
+        </is>
+      </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>402787699623</t>
+          <t>155034392297</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>huihuibest</t>
+          <t>Unbranded</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>4 Heads Chandelier Vintage Pendant Light Steampunk Style Loft Ceiling Fixture</t>
+          <t>E27 Ceiling Rose Light Fitting Vintage Industrial Pendant Holder</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>88+</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>GBP  69.12</t>
+          <t>GBP  8.99</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>99.8% (9.6K)</t>
+          <t>99.7% (5.5K)</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -3261,50 +3123,58 @@
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr"/>
-      <c r="M33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Lamp Holder, Bulb Holder, E27 Holder</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>Ceiling Rose Lamp Holder, Pendant Lamp Holder, Bakelite Bulb Holder, E27 Fitting</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>E27 Vintage Bakelite Pendant Lamp Holder with Cord Grip, Ceiling Rose Bulb Holder Kit, Screw E27 Fitting with Switch</t>
+        </is>
+      </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: huihuibest</t>
+          <t>Competitor seller: theyinltd</t>
         </is>
       </c>
     </row>
     <row r="34" ht="52" customHeight="1">
       <c r="A34" s="2" t="inlineStr"/>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Bulbs</t>
-        </is>
-      </c>
+      <c r="B34" s="2" t="inlineStr"/>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>223224109836</t>
+          <t>396977702027</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Auraglow</t>
+          <t>Luxa</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Auraglow Mysa LED Light Bulb Vintage Retro Edison Style Decorative E27 T30 Tube</t>
+          <t>Black Retro E27 Vintage Screw In Light Bulb Lamp Holder Ceiling Rose</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>38</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>GBP  10.99</t>
+          <t>GBP  8.99</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>99.8% (188.5K)</t>
+          <t>100% (2.5K)</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -3312,25 +3182,17 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr"/>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>LED Bulb, Filament Bulb, Light Bulb</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>Edison Bulb, Vintage LED Bulb, E27 Bulb, Dimmable LED Filament Bulb</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="inlineStr">
-        <is>
-          <t>E27 Vintage Edison LED Filament Bulb Warm White, Dimmable Squirrel Cage Light Bulb, ST64 Amber Decorative LED Bulb 4W</t>
-        </is>
-      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Save up to 5% Multi-buy</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr"/>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: safield-online</t>
+          <t>Competitor seller: gmuk.ltd</t>
         </is>
       </c>
     </row>
@@ -3339,7 +3201,7 @@
       <c r="B35" s="2" t="inlineStr"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>142340181955</t>
+          <t>363478927381</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -3349,22 +3211,22 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Vintage Edison Filament LED Bulb Teardrop E27 ES 4W Clear Warm White Dimmable</t>
+          <t>1x Brass Rose Ceiling Pendant Light Kit 1 Metre Flex ES E27</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>GBP  3.50</t>
+          <t>GBP  4.99</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>99.8% (22.6K)</t>
+          <t>99.6% (185.3K)</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -3372,13 +3234,17 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Save up to 8% Multi-buy</t>
+        </is>
+      </c>
       <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="2" t="inlineStr"/>
       <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: thelampfactoryuk</t>
+          <t>Competitor seller: dqpltd</t>
         </is>
       </c>
     </row>
@@ -3387,32 +3253,32 @@
       <c r="B36" s="2" t="inlineStr"/>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>352802795272</t>
+          <t>322867838398</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>ValueLights</t>
+          <t>Unbranded</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Filament LED Light Bulb Decorative Vintage Edison Lightbulb</t>
+          <t>CERTIFIED ES E27 Ceiling Rose Chain Pendant Lamp Holder Kit UK</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>102+</t>
+          <t>28+</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>GBP  5.99 to 19.99</t>
+          <t>GBP  99.00</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>99.8% (685K)</t>
+          <t>100% (12.6K)</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -3420,17 +3286,13 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>Save up to 15% Multi-buy</t>
-        </is>
-      </c>
+      <c r="J36" s="2" t="inlineStr"/>
       <c r="K36" s="2" t="inlineStr"/>
       <c r="L36" s="2" t="inlineStr"/>
       <c r="M36" s="2" t="inlineStr"/>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: value-lights</t>
+          <t>Competitor seller: ediscount247</t>
         </is>
       </c>
     </row>
@@ -3439,32 +3301,32 @@
       <c r="B37" s="2" t="inlineStr"/>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>353725905176</t>
+          <t>283939294098</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Kanlux</t>
+          <t>Crown Lighting</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>10x EXTRA LARGE GLOBE FILAMENT E27 BULB Vintage Incandescent Edison</t>
+          <t>E27 Chrome Ceiling Rose Pendant With Tube And Lamp Holder Fitting</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>GBP  70.94</t>
+          <t>GBP  29.95</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>99.7% (84.9K)</t>
+          <t>100% (8.5K)</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -3478,318 +3340,6 @@
       <c r="M37" s="2" t="inlineStr"/>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: auctionzltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="52" customHeight="1">
-      <c r="A38" s="2" t="inlineStr"/>
-      <c r="B38" s="2" t="inlineStr"/>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>364884514396</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>Unbranded</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>2x 4W (=33W) Vintage T30 Tube Gold LED Filament ES E27 2700K Light Bulbs</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>GBP  9.99</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>99.6% (185.3K)</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>With postage</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>Save up to 8% Multi-buy</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="inlineStr"/>
-      <c r="L38" s="2" t="inlineStr"/>
-      <c r="M38" s="2" t="inlineStr"/>
-      <c r="N38" s="2" t="inlineStr">
-        <is>
-          <t>Competitor seller: dqpltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="52" customHeight="1">
-      <c r="A39" s="2" t="inlineStr"/>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Lamp Holder</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>396977702027</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>Luxa</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>Black Retro E27 Vintage Screw In Light Bulb Lamp Holder Ceiling Rose Pendant Kit</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>GBP  8.99</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>100% (2.5K)</t>
-        </is>
-      </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>With postage</t>
-        </is>
-      </c>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>Save up to 5% Multi-buy</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="inlineStr">
-        <is>
-          <t>Lamp Holder, Bulb Holder, E27 Holder</t>
-        </is>
-      </c>
-      <c r="L39" s="2" t="inlineStr">
-        <is>
-          <t>Ceiling Rose Lamp Holder, Pendant Lamp Holder, Bakelite Bulb Holder, E27 Fitting</t>
-        </is>
-      </c>
-      <c r="M39" s="2" t="inlineStr">
-        <is>
-          <t>E27 Vintage Bakelite Pendant Lamp Holder with Cord Grip, Ceiling Rose Bulb Holder Kit, Screw E27 Fitting with Switch</t>
-        </is>
-      </c>
-      <c r="N39" s="2" t="inlineStr">
-        <is>
-          <t>Competitor seller: gmuk.ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="52" customHeight="1">
-      <c r="A40" s="2" t="inlineStr"/>
-      <c r="B40" s="2" t="inlineStr"/>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>184848546669</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>Knightsbridge</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>ES E27 Screw In Bulb Lamp Matt White Pendant Set Lampholder Ceiling Rose</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>GBP  18.99</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>99.9% (44.1K)</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>With postage</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="inlineStr"/>
-      <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr"/>
-      <c r="M40" s="2" t="inlineStr"/>
-      <c r="N40" s="2" t="inlineStr">
-        <is>
-          <t>Competitor seller: colchester-electrical-wholesale</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="52" customHeight="1">
-      <c r="A41" s="2" t="inlineStr"/>
-      <c r="B41" s="2" t="inlineStr"/>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>224707047105</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>Unbranded</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>E27 Ceiling Rose Light Fitting Vintage Industrial Flex Pendant Lamp Bulb Holder</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>GBP  10.59</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>99.6% (2.9K)</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>Free postage</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr"/>
-      <c r="K41" s="2" t="inlineStr"/>
-      <c r="L41" s="2" t="inlineStr"/>
-      <c r="M41" s="2" t="inlineStr"/>
-      <c r="N41" s="2" t="inlineStr">
-        <is>
-          <t>Competitor seller: yuki-store-2020</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="52" customHeight="1">
-      <c r="A42" s="2" t="inlineStr"/>
-      <c r="B42" s="2" t="inlineStr"/>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>225227368158</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Crown</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>E27 Ceiling Rose Pendant With Tube And Lamp Holder Brass Light Fitting UK</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>GBP  18.85</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>100% (1.2K)</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>With postage</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr"/>
-      <c r="K42" s="2" t="inlineStr"/>
-      <c r="L42" s="2" t="inlineStr"/>
-      <c r="M42" s="2" t="inlineStr"/>
-      <c r="N42" s="2" t="inlineStr">
-        <is>
-          <t>Competitor seller: universalmerchandise4u</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="52" customHeight="1">
-      <c r="A43" s="2" t="inlineStr"/>
-      <c r="B43" s="2" t="inlineStr"/>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>274419951502</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Crown Lighting</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>E27 Modern Ceiling Rose Pendant With Tube And Lamp Holder Fitting</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>GBP  24.95</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>100% (8.5K)</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>With postage</t>
-        </is>
-      </c>
-      <c r="J43" s="2" t="inlineStr"/>
-      <c r="K43" s="2" t="inlineStr"/>
-      <c r="L43" s="2" t="inlineStr"/>
-      <c r="M43" s="2" t="inlineStr"/>
-      <c r="N43" s="2" t="inlineStr">
-        <is>
           <t>Competitor seller: bandhstore</t>
         </is>
       </c>

</xml_diff>

<commit_message>
feat(eckr): 5 UK competitors per category (45 rows) - filled Cage/Spider/Pipe
Cage +1 (value-lights geometric); Spider +4 (loopsdirect/ThatCable,
nationallighting, themiddleaisleuk23, mossodor); Pipe +4 (industrial_cafe/
Moonlight Retail x4). All UK-verified. Thin niches filled with UK sellers that
don't all show a sold count (eBay only shows sold with recent sales).
Rebuilt dashboard/static/xlsx; re-published ph_task 496-499 (111847).
</commit_message>
<xml_diff>
--- a/development/abiraj_mini_aios_workbench/projects/PRJ-2026-017_ebay-competitor-keyword-research/evidence/final_outputs/REQ-20_ebay-competitor-keyword-research/REQ-20-D01_ebay_competitor_keyword_FINAL.xlsx
+++ b/development/abiraj_mini_aios_workbench/projects/PRJ-2026-017_ebay-competitor-keyword-research/evidence/final_outputs/REQ-20_ebay-competitor-keyword-research/REQ-20-D01_ebay_competitor_keyword_FINAL.xlsx
@@ -1031,6 +1031,231 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId36"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId37"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId38"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId39"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>41</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="41" name="Image 41" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId41"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>42</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="42" name="Image 42" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId42"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>43</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="43" name="Image 43" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId43"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>44</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="44" name="Image 44" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId44"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="45" name="Image 45" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId45"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1333,7 +1558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:N46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2538,39 +2763,31 @@
     </row>
     <row r="23" ht="52" customHeight="1">
       <c r="A23" s="2" t="inlineStr"/>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Cage pendant light</t>
-        </is>
-      </c>
+      <c r="B23" s="2" t="inlineStr"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>372257190104</t>
+          <t>372474939568</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>ValueLights</t>
+          <t>ThatCable</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Ceiling Light Shade Geometric Pendant Lampshade Industrial</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>429+</t>
-        </is>
-      </c>
+          <t>Multi Light Ceiling Pendant 6 Bulb Gloss Copper Industrial Adjustable</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>GBP  12.99 to 15.99</t>
+          <t>GBP  94.99</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>99.8% (685K)</t>
+          <t>98.3% (235.1K)</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -2578,29 +2795,13 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>Save up to 10% Multi-buy</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>Cage Pendant Light, Cage Light, Metal Cage Pendant</t>
-        </is>
-      </c>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>Industrial Cage Light, Wire Cage Pendant, Vintage Cage Lamp, Cage Ceiling Light</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="inlineStr">
-        <is>
-          <t>Black Metal Cage Pendant Light for Kitchen, Industrial Wire Cage Hanging Lamp E27, Vintage Cage Ceiling Light Fitting</t>
-        </is>
-      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: value-lights</t>
+          <t>Competitor seller: loopsdirect</t>
         </is>
       </c>
     </row>
@@ -2609,32 +2810,28 @@
       <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>232708905363</t>
+          <t>303227195662</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>ValueLights</t>
+          <t>National Lighting</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Industrial Metal Ceiling Pendant Light Shade Easy Fit</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>289+</t>
-        </is>
-      </c>
+          <t>Adjustable Pendant Light Fitting Ceiling Rose E27 Industrial Spider</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>GBP  22.99 to 25.99</t>
+          <t>GBP  13.42 to 59.92</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>99.8% (685K)</t>
+          <t>99.6% (18.4K)</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -2642,17 +2839,13 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>From GBP 20.69 with coupon</t>
-        </is>
-      </c>
+      <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: value-lights</t>
+          <t>Competitor seller: nationallighting</t>
         </is>
       </c>
     </row>
@@ -2661,32 +2854,28 @@
       <c r="B25" s="2" t="inlineStr"/>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>131173303482</t>
+          <t>317136278633</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>(not listed)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Black Wire Cage Light Shade Steel E27 Industrial Pendant</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>252</t>
-        </is>
-      </c>
+          <t>6 Light Spider Pendant Ceiling Light Hemp Rope Industrial Multiple Hanging</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>GBP  13.00</t>
+          <t>GBP  68.98</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>99.8% (22.6K)</t>
+          <t>99.3% (4.7K)</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -2694,13 +2883,17 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Save up to 15% Multi-buy</t>
+        </is>
+      </c>
       <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: thelampfactoryuk</t>
+          <t>Competitor seller: themiddleaisleuk23</t>
         </is>
       </c>
     </row>
@@ -2709,32 +2902,28 @@
       <c r="B26" s="2" t="inlineStr"/>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>141264804458</t>
+          <t>166809932104</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>Mossodor</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Bronze Wire Cage Light Shade Steel E27 Industrial Pendant</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>157</t>
-        </is>
-      </c>
+          <t>Black Pendant Light Industrial Ceiling Light Spider Modern Cluster E27</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>GBP  13.00</t>
+          <t>GBP  32.95</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>99.8% (22.6K)</t>
+          <t>98.3% (886)</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2742,13 +2931,17 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Save up to 20% Multi-buy</t>
+        </is>
+      </c>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: thelampfactoryuk</t>
+          <t>Competitor seller: mossodor_lighting</t>
         </is>
       </c>
     </row>
@@ -2756,37 +2949,37 @@
       <c r="A27" s="2" t="inlineStr"/>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Pipe Light</t>
+          <t>Cage pendant light</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>262744851290</t>
+          <t>372257190104</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>(not listed)</t>
+          <t>ValueLights</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Silver Industrial Ceiling Light Vintage Antique Pendant Pipe Cage</t>
+          <t>Ceiling Light Shade Geometric Pendant Lampshade Industrial</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>429+</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>GBP  46.99</t>
+          <t>GBP  12.99 to 15.99</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>98.5% (15.2K)</t>
+          <t>99.8% (685K)</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -2794,63 +2987,63 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Save up to 10% Multi-buy</t>
+        </is>
+      </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Pipe Light, Pipe Pendant Light, Steampunk Light</t>
+          <t>Cage Pendant Light, Cage Light, Metal Cage Pendant</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Industrial Pipe Light, Steampunk Pendant, Pipe Wall Light, Water Pipe Lamp</t>
+          <t>Industrial Cage Light, Wire Cage Pendant, Vintage Cage Lamp, Cage Ceiling Light</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Industrial Steampunk Pipe Pendant Light for Kitchen Island, Black Metal Pipe Ceiling Light E27, Vintage Water Pipe Wall Lamp</t>
+          <t>Black Metal Cage Pendant Light for Kitchen, Industrial Wire Cage Hanging Lamp E27, Vintage Cage Ceiling Light Fitting</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: sj_modern_antiques</t>
+          <t>Competitor seller: value-lights</t>
         </is>
       </c>
     </row>
     <row r="28" ht="52" customHeight="1">
       <c r="A28" s="2" t="inlineStr"/>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Bulbs</t>
-        </is>
-      </c>
+      <c r="B28" s="2" t="inlineStr"/>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>303695648760</t>
+          <t>232708905363</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Kanlux</t>
+          <t>ValueLights</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>2x Vintage Filament LED Edison Screw Bulb E27 Decorative ST64</t>
+          <t>Industrial Metal Ceiling Pendant Light Shade Easy Fit</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>237</t>
+          <t>289+</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>GBP  16.95</t>
+          <t>GBP  22.99 to 25.99</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>99.7% (84.9K)</t>
+          <t>99.8% (685K)</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2860,27 +3053,15 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Save up to 20% Multi-buy</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>LED Bulb, Filament Bulb, Light Bulb</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>Edison Bulb, Vintage LED Bulb, E27 Bulb, Dimmable LED Filament Bulb</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr">
-        <is>
-          <t>E27 Vintage Edison LED Filament Bulb Warm White, Dimmable Squirrel Cage Light Bulb, ST64 Amber Decorative LED Bulb 4W</t>
-        </is>
-      </c>
+          <t>From GBP 20.69 with coupon</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: auctionzltd</t>
+          <t>Competitor seller: value-lights</t>
         </is>
       </c>
     </row>
@@ -2889,32 +3070,32 @@
       <c r="B29" s="2" t="inlineStr"/>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>223224109836</t>
+          <t>131173303482</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Auraglow</t>
+          <t>Unbranded</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Auraglow Mysa LED Light Bulb Vintage Retro Edison Style E27 T30</t>
+          <t>Black Wire Cage Light Shade Steel E27 Industrial Pendant</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>252</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>GBP  10.99</t>
+          <t>GBP  13.00</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>99.8% (188.5K)</t>
+          <t>99.8% (22.6K)</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -2928,7 +3109,7 @@
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: safield-online</t>
+          <t>Competitor seller: thelampfactoryuk</t>
         </is>
       </c>
     </row>
@@ -2937,7 +3118,7 @@
       <c r="B30" s="2" t="inlineStr"/>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>142340181955</t>
+          <t>141264804458</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2947,17 +3128,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Vintage Edison Filament LED Bulb Teardrop E27 ES 4W Warm White</t>
+          <t>Bronze Wire Cage Light Shade Steel E27 Industrial Pendant</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>157</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>GBP  3.50</t>
+          <t>GBP  13.00</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2985,32 +3166,32 @@
       <c r="B31" s="2" t="inlineStr"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>193185894331</t>
+          <t>372864053966</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Auraglow</t>
+          <t>ValueLights</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Auraglow Mysa LED Light Bulb Vintage Retro Edison Style G125 Globe</t>
+          <t>Geometric Globe Lampshade Metal Pendant Ceiling Light Shade</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>156+</t>
+          <t>125+</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>GBP  16.99</t>
+          <t>GBP  14.99 to 17.99</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>99.8% (188.5K)</t>
+          <t>99.8% (685K)</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -3018,47 +3199,55 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>10% off</t>
+        </is>
+      </c>
       <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: safield-online</t>
+          <t>Competitor seller: value-lights</t>
         </is>
       </c>
     </row>
     <row r="32" ht="52" customHeight="1">
       <c r="A32" s="2" t="inlineStr"/>
-      <c r="B32" s="2" t="inlineStr"/>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Pipe Light</t>
+        </is>
+      </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>353206988280</t>
+          <t>262744851290</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Kanlux</t>
+          <t>(not listed)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>E27 LED Vintage Edison Spiral Filament Industrial Bulb Amber</t>
+          <t>Silver Industrial Ceiling Light Vintage Antique Pendant Pipe Cage</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>114</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>GBP  7.95</t>
+          <t>GBP  46.99</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>99.7% (84.9K)</t>
+          <t>98.5% (15.2K)</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -3066,55 +3255,55 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>Save up to 12% Multi-buy</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr"/>
-      <c r="M32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Pipe Light, Pipe Pendant Light, Steampunk Light</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Industrial Pipe Light, Steampunk Pendant, Pipe Wall Light, Water Pipe Lamp</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Industrial Steampunk Pipe Pendant Light for Kitchen Island, Black Metal Pipe Ceiling Light E27, Vintage Water Pipe Wall Lamp</t>
+        </is>
+      </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: auctionzltd</t>
+          <t>Competitor seller: sj_modern_antiques</t>
         </is>
       </c>
     </row>
     <row r="33" ht="52" customHeight="1">
       <c r="A33" s="2" t="inlineStr"/>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Lamp Holder</t>
-        </is>
-      </c>
+      <c r="B33" s="2" t="inlineStr"/>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>155034392297</t>
+          <t>236319831602</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>Moonlight Retail</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>E27 Ceiling Rose Light Fitting Vintage Industrial Pendant Holder</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>88+</t>
-        </is>
-      </c>
+          <t>Industrial Vintage Ceiling Lights Metal Pipe Retro Loft Pendant Steampunk</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>GBP  8.99</t>
+          <t>GBP  36.95 to 53.75</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>99.7% (5.5K)</t>
+          <t>100% (1.1K)</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -3123,24 +3312,12 @@
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>Lamp Holder, Bulb Holder, E27 Holder</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>Ceiling Rose Lamp Holder, Pendant Lamp Holder, Bakelite Bulb Holder, E27 Fitting</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="inlineStr">
-        <is>
-          <t>E27 Vintage Bakelite Pendant Lamp Holder with Cord Grip, Ceiling Rose Bulb Holder Kit, Screw E27 Fitting with Switch</t>
-        </is>
-      </c>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr"/>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: theyinltd</t>
+          <t>Competitor seller: industrial_cafe</t>
         </is>
       </c>
     </row>
@@ -3149,32 +3326,28 @@
       <c r="B34" s="2" t="inlineStr"/>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>396977702027</t>
+          <t>236319380461</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Luxa</t>
+          <t>Moonlight Retail</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Black Retro E27 Vintage Screw In Light Bulb Lamp Holder Ceiling Rose</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
-      </c>
+          <t>Industrial Steampunk Lighting Iron Pipe Edison Bulb Ceiling Bar Light Rope</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>GBP  8.99</t>
+          <t>GBP  67.19 to 77.27</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>100% (2.5K)</t>
+          <t>100% (1.1K)</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -3182,17 +3355,13 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>Save up to 5% Multi-buy</t>
-        </is>
-      </c>
+      <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr"/>
       <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr"/>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: gmuk.ltd</t>
+          <t>Competitor seller: industrial_cafe</t>
         </is>
       </c>
     </row>
@@ -3201,32 +3370,28 @@
       <c r="B35" s="2" t="inlineStr"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>363478927381</t>
+          <t>336171618850</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>Moonlight Retail</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>1x Brass Rose Ceiling Pendant Light Kit 1 Metre Flex ES E27</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
+          <t>Industrial Steampunk Chandelier Iron Pipe Edison Bulb Ceiling Bar Light</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>GBP  4.99</t>
+          <t>GBP  167.99 to 250.87</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>99.6% (185.3K)</t>
+          <t>100% (1.1K)</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -3234,17 +3399,13 @@
           <t>With postage</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>Save up to 8% Multi-buy</t>
-        </is>
-      </c>
+      <c r="J35" s="2" t="inlineStr"/>
       <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="2" t="inlineStr"/>
       <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: dqpltd</t>
+          <t>Competitor seller: industrial_cafe</t>
         </is>
       </c>
     </row>
@@ -3253,32 +3414,28 @@
       <c r="B36" s="2" t="inlineStr"/>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>322867838398</t>
+          <t>336163640353</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>Moonlight Retail</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>CERTIFIED ES E27 Ceiling Rose Chain Pendant Lamp Holder Kit UK</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>28+</t>
-        </is>
-      </c>
+          <t>Industrial Steampunk Light Iron Pipe Edison Bulb Ceiling Chain 7 Heads</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>GBP  99.00</t>
+          <t>GBP  101.91</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>100% (12.6K)</t>
+          <t>100% (1.1K)</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -3292,53 +3449,533 @@
       <c r="M36" s="2" t="inlineStr"/>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: ediscount247</t>
+          <t>Competitor seller: industrial_cafe</t>
         </is>
       </c>
     </row>
     <row r="37" ht="52" customHeight="1">
       <c r="A37" s="2" t="inlineStr"/>
-      <c r="B37" s="2" t="inlineStr"/>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Bulbs</t>
+        </is>
+      </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
+          <t>303695648760</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Kanlux</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>2x Vintage Filament LED Edison Screw Bulb E27 Decorative ST64</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>237</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>GBP  16.95</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>99.7% (84.9K)</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>With postage</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Save up to 20% Multi-buy</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>LED Bulb, Filament Bulb, Light Bulb</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Edison Bulb, Vintage LED Bulb, E27 Bulb, Dimmable LED Filament Bulb</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>E27 Vintage Edison LED Filament Bulb Warm White, Dimmable Squirrel Cage Light Bulb, ST64 Amber Decorative LED Bulb 4W</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>Competitor seller: auctionzltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="52" customHeight="1">
+      <c r="A38" s="2" t="inlineStr"/>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>223224109836</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Auraglow</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Auraglow Mysa LED Light Bulb Vintage Retro Edison Style E27 T30</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>GBP  10.99</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>99.8% (188.5K)</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>With postage</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>Competitor seller: safield-online</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="52" customHeight="1">
+      <c r="A39" s="2" t="inlineStr"/>
+      <c r="B39" s="2" t="inlineStr"/>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>142340181955</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Unbranded</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Vintage Edison Filament LED Bulb Teardrop E27 ES 4W Warm White</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>169</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>GBP  3.50</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>99.8% (22.6K)</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>With postage</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr"/>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>Competitor seller: thelampfactoryuk</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="52" customHeight="1">
+      <c r="A40" s="2" t="inlineStr"/>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>193185894331</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Auraglow</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Auraglow Mysa LED Light Bulb Vintage Retro Edison Style G125 Globe</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>156+</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>GBP  16.99</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>99.8% (188.5K)</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>With postage</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>Competitor seller: safield-online</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="52" customHeight="1">
+      <c r="A41" s="2" t="inlineStr"/>
+      <c r="B41" s="2" t="inlineStr"/>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>353206988280</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Kanlux</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>E27 LED Vintage Edison Spiral Filament Industrial Bulb Amber</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>GBP  7.95</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>99.7% (84.9K)</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>With postage</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Save up to 12% Multi-buy</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr"/>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>Competitor seller: auctionzltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="52" customHeight="1">
+      <c r="A42" s="2" t="inlineStr"/>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Lamp Holder</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>155034392297</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Unbranded</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>E27 Ceiling Rose Light Fitting Vintage Industrial Pendant Holder</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>88+</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>GBP  8.99</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>99.7% (5.5K)</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>With postage</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Lamp Holder, Bulb Holder, E27 Holder</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Ceiling Rose Lamp Holder, Pendant Lamp Holder, Bakelite Bulb Holder, E27 Fitting</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>E27 Vintage Bakelite Pendant Lamp Holder with Cord Grip, Ceiling Rose Bulb Holder Kit, Screw E27 Fitting with Switch</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>Competitor seller: theyinltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="52" customHeight="1">
+      <c r="A43" s="2" t="inlineStr"/>
+      <c r="B43" s="2" t="inlineStr"/>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>396977702027</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Luxa</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Black Retro E27 Vintage Screw In Light Bulb Lamp Holder Ceiling Rose</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>GBP  8.99</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>100% (2.5K)</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>With postage</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Save up to 5% Multi-buy</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr"/>
+      <c r="M43" s="2" t="inlineStr"/>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>Competitor seller: gmuk.ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="52" customHeight="1">
+      <c r="A44" s="2" t="inlineStr"/>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>363478927381</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Unbranded</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>1x Brass Rose Ceiling Pendant Light Kit 1 Metre Flex ES E27</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>GBP  4.99</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>99.6% (185.3K)</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>With postage</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Save up to 8% Multi-buy</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr"/>
+      <c r="M44" s="2" t="inlineStr"/>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>Competitor seller: dqpltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="52" customHeight="1">
+      <c r="A45" s="2" t="inlineStr"/>
+      <c r="B45" s="2" t="inlineStr"/>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>322867838398</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Unbranded</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>CERTIFIED ES E27 Ceiling Rose Chain Pendant Lamp Holder Kit UK</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>28+</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>GBP  99.00</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>100% (12.6K)</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>With postage</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr"/>
+      <c r="L45" s="2" t="inlineStr"/>
+      <c r="M45" s="2" t="inlineStr"/>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>Competitor seller: ediscount247</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="52" customHeight="1">
+      <c r="A46" s="2" t="inlineStr"/>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
           <t>283939294098</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>Crown Lighting</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>E27 Chrome Ceiling Rose Pendant With Tube And Lamp Holder Fitting</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>GBP  29.95</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>100% (8.5K)</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>With postage</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr"/>
-      <c r="K37" s="2" t="inlineStr"/>
-      <c r="L37" s="2" t="inlineStr"/>
-      <c r="M37" s="2" t="inlineStr"/>
-      <c r="N37" s="2" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>With postage</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr"/>
+      <c r="M46" s="2" t="inlineStr"/>
+      <c r="N46" s="2" t="inlineStr">
         <is>
           <t>Competitor seller: bandhstore</t>
         </is>

</xml_diff>